<commit_message>
fix: align import example template headers
</commit_message>
<xml_diff>
--- a/public/templates/we-discipline-first-client-bulk-import.xlsx
+++ b/public/templates/we-discipline-first-client-bulk-import.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Membres" sheetId="1" r:id="R503161b931cc4487"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exemple" sheetId="2" r:id="R2f39ad2feb4d47ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="References" sheetId="3" r:id="R8806ada402b546eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aide" sheetId="4" r:id="R84ff395720534327"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compatibilite" sheetId="5" r:id="Rb54b6c6536ff4bcd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Membres" sheetId="1" r:id="Rfca5d81552fb4ab3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exemple" sheetId="2" r:id="R632e5fde0b254596"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="References" sheetId="3" r:id="R123b93b5e9e5437d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aide" sheetId="4" r:id="Re68c517bef3e43ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compatibilite" sheetId="5" r:id="Rd8e3608b8bd04df5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -451,123 +451,75 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A1" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Code membre auto (laisser vide)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B1" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Prenom</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C1" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Nom</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D1" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Type membre</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E1" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Telephone</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F1" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Email</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G1" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Date naissance</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H1" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Adresse</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I1" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Nom parent</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J1" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Telephone parent</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K1" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Date inscription</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L1" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Groupe</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M1" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Formule</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N1" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Debut groupe</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O1" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Debut abonnement</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P1" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Fin abonnement</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q1" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Montant total</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R1" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Deja paye</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S1" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Seances restantes</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="T1" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Date paiement</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="U1" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Mode paiement</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="V1" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Note reprise</x:t>
-        </x:is>
+      <x:c r="A1" s="5" t="str">
+        <x:v>Code membre auto (laisser vide)</x:v>
+      </x:c>
+      <x:c r="B1" s="5" t="str">
+        <x:v>Prénom</x:v>
+      </x:c>
+      <x:c r="C1" s="5" t="str">
+        <x:v>Nom</x:v>
+      </x:c>
+      <x:c r="D1" s="5" t="str">
+        <x:v>Type membre</x:v>
+      </x:c>
+      <x:c r="E1" s="5" t="str">
+        <x:v>Téléphone</x:v>
+      </x:c>
+      <x:c r="F1" s="5" t="str">
+        <x:v>Email</x:v>
+      </x:c>
+      <x:c r="G1" s="5" t="str">
+        <x:v>Date naissance</x:v>
+      </x:c>
+      <x:c r="H1" s="5" t="str">
+        <x:v>Adresse</x:v>
+      </x:c>
+      <x:c r="I1" s="5" t="str">
+        <x:v>Nom parent</x:v>
+      </x:c>
+      <x:c r="J1" s="5" t="str">
+        <x:v>Téléphone parent</x:v>
+      </x:c>
+      <x:c r="K1" s="5" t="str">
+        <x:v>Date inscription</x:v>
+      </x:c>
+      <x:c r="L1" s="5" t="str">
+        <x:v>Groupe</x:v>
+      </x:c>
+      <x:c r="M1" s="5" t="str">
+        <x:v>Formule</x:v>
+      </x:c>
+      <x:c r="N1" s="5" t="str">
+        <x:v>Début groupe</x:v>
+      </x:c>
+      <x:c r="O1" s="5" t="str">
+        <x:v>Début abonnement</x:v>
+      </x:c>
+      <x:c r="P1" s="5" t="str">
+        <x:v>Fin abonnement</x:v>
+      </x:c>
+      <x:c r="Q1" s="5" t="str">
+        <x:v>Montant total</x:v>
+      </x:c>
+      <x:c r="R1" s="5" t="str">
+        <x:v>Déjà payé</x:v>
+      </x:c>
+      <x:c r="S1" s="5" t="str">
+        <x:v>Séances restantes</x:v>
+      </x:c>
+      <x:c r="T1" s="5" t="str">
+        <x:v>Date paiement</x:v>
+      </x:c>
+      <x:c r="U1" s="5" t="str">
+        <x:v>Mode paiement</x:v>
+      </x:c>
+      <x:c r="V1" s="5" t="str">
+        <x:v>Note reprise</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">M001-amineclient-9999</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="A2" s="7"/>
       <x:c r="B2" s="7" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Amine</x:t>
@@ -649,11 +601,7 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">M002-nourclient-8888</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="A3" s="7"/>
       <x:c r="B3" s="7" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Nour</x:t>

</xml_diff>